<commit_message>
Publish course materials (2360611)
Generated by scripts/publish_student.py from the source repository at 2360611: "publish_student: never delete a student's .venv"
</commit_message>
<xml_diff>
--- a/schedule/CSCI3495_schedule_fall2026.xlsx
+++ b/schedule/CSCI3495_schedule_fall2026.xlsx
@@ -148,16 +148,20 @@
     <t>Wed Sep 9</t>
   </si>
   <si>
-    <t>Python, NumPy, Pandas, Seaborn, Scikit-Learn</t>
+    <t>Python for NLP: comprehensions and Counter; NumPy shape, dtype, broadcasting</t>
   </si>
   <si>
     <t>Lecture, Coding</t>
   </si>
   <si>
-    <t>Watch: Complete Python NumPy Tutorial (Keith Galli, 58 min)</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=GB9ByFAIAH4</t>
+    <t>Watch 5 short videos (~50 min total): Python basics (Indently, 10:30); NumPy (Bro Code, 5:07); pandas (Python Programmer, 13:31); seaborn (Kimberly Fessel, 7:26); PyTorch (LeakyAI, 13:11)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=fWjsdhR3z3c
+https://www.youtube.com/watch?v=Gc-dwloxNFE
+https://www.youtube.com/watch?v=iGFdh6_FePU
+https://www.youtube.com/watch?v=vaf4ir8eT38
+https://www.youtube.com/watch?v=r5D6bnCJ490</t>
   </si>
   <si>
     <t>Last day to opt Pass/Fail/Audit (Sep 11)</t>
@@ -166,7 +170,7 @@
     <t>Mon Sep 14</t>
   </si>
   <si>
-    <t>PyTorch: autograd &amp; backpropagation</t>
+    <t>pandas &amp; PyTorch tensors: DataFrames, groupby, plotting; tensor shapes and autograd</t>
   </si>
   <si>
     <t>Lecture, Quiz, Coding</t>
@@ -246,7 +250,7 @@
     <t>Wed Sep 30</t>
   </si>
   <si>
-    <t>Attention &amp; Transformer</t>
+    <t>Seq2seq &amp; attention: encoder-decoder and the attention mechanism</t>
   </si>
   <si>
     <t>HW2 due</t>
@@ -255,10 +259,7 @@
     <t>Mon Oct 5</t>
   </si>
   <si>
-    <t>Whiteboard &amp; Project Proposal</t>
-  </si>
-  <si>
-    <t>Whiteboard, Project-Time</t>
+    <t>The Transformer: self-attention, multi-head, positional encoding</t>
   </si>
   <si>
     <t>Read 'Attention Is All You Need' (Vaswani 2017)</t>
@@ -279,10 +280,10 @@
     <t>Wed Oct 7</t>
   </si>
   <si>
-    <t>Contextual representations &amp; transfer learning: ELMo; pretrain→finetune</t>
-  </si>
-  <si>
-    <t>Lecture, Discussion</t>
+    <t>BERT - Conceptual</t>
+  </si>
+  <si>
+    <t>Lecture, Whiteboard</t>
   </si>
   <si>
     <t>HW3 released</t>
@@ -291,7 +292,7 @@
     <t>Mon Oct 12</t>
   </si>
   <si>
-    <t>BERT &amp; masked language modeling: bidirectional pretraining, fine-tuning</t>
+    <t>BERT - Programming</t>
   </si>
   <si>
     <t>Read BERT (Devlin 2019)</t>
@@ -404,6 +405,9 @@
   </si>
   <si>
     <t>In-context learning &amp; prompt-engineering foundations: zero/few-shot</t>
+  </si>
+  <si>
+    <t>Lecture, Discussion</t>
   </si>
   <si>
     <t>Prepare the checkpoint talk</t>
@@ -1249,7 +1253,7 @@
       </c>
       <c r="J4" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="28.5" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="70" customFormat="1" s="5">
       <c r="A5" s="8">
         <v>2</v>
       </c>
@@ -1279,7 +1283,7 @@
         <v>31</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="51">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="70">
       <c r="A6" s="13"/>
       <c r="B6" s="14"/>
       <c r="C6" s="10" t="s">
@@ -1303,7 +1307,7 @@
       </c>
       <c r="J6" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="20.25" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="24" customFormat="1" s="5">
       <c r="A7" s="16"/>
       <c r="B7" s="17" t="s">
         <v>38</v>
@@ -1321,7 +1325,7 @@
       <c r="I7" s="18"/>
       <c r="J7" s="18"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="39.75" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="84" customFormat="1" s="5">
       <c r="A8" s="8">
         <v>3</v>
       </c>
@@ -1349,7 +1353,7 @@
         <v>47</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="39.75">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="58">
       <c r="A9" s="13"/>
       <c r="B9" s="14"/>
       <c r="C9" s="10" t="s">
@@ -1371,7 +1375,7 @@
       </c>
       <c r="J9" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="28.5" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="58" customFormat="1" s="5">
       <c r="A10" s="8">
         <v>4</v>
       </c>
@@ -1393,7 +1397,7 @@
       <c r="I10" s="11"/>
       <c r="J10" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="45">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="84">
       <c r="A11" s="13"/>
       <c r="B11" s="14"/>
       <c r="C11" s="10" t="s">
@@ -1445,7 +1449,7 @@
         <v>67</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="84">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="45">
       <c r="A13" s="13"/>
       <c r="B13" s="14"/>
       <c r="C13" s="10" t="s">
@@ -1469,7 +1473,7 @@
       </c>
       <c r="J13" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="58" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="39.75" customFormat="1" s="5">
       <c r="A14" s="8">
         <v>6</v>
       </c>
@@ -1483,7 +1487,7 @@
         <v>75</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F14" s="11"/>
       <c r="G14" s="11"/>
@@ -1493,7 +1497,7 @@
       <c r="I14" s="11"/>
       <c r="J14" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="70">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="39.75">
       <c r="A15" s="13"/>
       <c r="B15" s="14"/>
       <c r="C15" s="10" t="s">
@@ -1503,67 +1507,67 @@
         <v>78</v>
       </c>
       <c r="E15" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="G15" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="G15" s="15" t="s">
+      <c r="H15" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="I15" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="I15" s="11" t="s">
-        <v>83</v>
-      </c>
       <c r="J15" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="58" customFormat="1" s="5">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="39.75" customFormat="1" s="5">
       <c r="A16" s="8">
         <v>7</v>
       </c>
       <c r="B16" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="D16" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="D16" s="11" t="s">
+      <c r="E16" s="11" t="s">
         <v>86</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>87</v>
       </c>
       <c r="F16" s="11"/>
       <c r="G16" s="11"/>
       <c r="H16" s="11" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I16" s="11"/>
       <c r="J16" s="11"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="70">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="39.75">
       <c r="A17" s="13"/>
       <c r="B17" s="14"/>
       <c r="C17" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" s="11" t="s">
         <v>89</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>90</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>50</v>
       </c>
       <c r="F17" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="G17" s="15" t="s">
         <v>91</v>
-      </c>
-      <c r="G17" s="15" t="s">
-        <v>92</v>
       </c>
       <c r="H17" s="11"/>
       <c r="I17" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J17" s="11"/>
     </row>
@@ -1572,39 +1576,39 @@
         <v>8</v>
       </c>
       <c r="B18" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C18" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="D18" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="D18" s="11" t="s">
+      <c r="E18" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="F18" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="E18" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="F18" s="11" t="s">
+      <c r="G18" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="G18" s="15" t="s">
+      <c r="H18" s="11" t="s">
         <v>98</v>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>99</v>
       </c>
       <c r="I18" s="11"/>
       <c r="J18" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="58">
       <c r="A19" s="13"/>
       <c r="B19" s="14"/>
       <c r="C19" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="D19" s="11" t="s">
         <v>101</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>102</v>
       </c>
       <c r="E19" s="11" t="s">
         <v>57</v>
@@ -1613,7 +1617,7 @@
       <c r="G19" s="11"/>
       <c r="H19" s="11"/>
       <c r="I19" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="J19" s="11"/>
     </row>
@@ -1622,13 +1626,13 @@
         <v>9</v>
       </c>
       <c r="B20" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="D20" s="11" t="s">
         <v>105</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>106</v>
       </c>
       <c r="E20" s="11" t="s">
         <v>65</v>
@@ -1636,34 +1640,34 @@
       <c r="F20" s="11"/>
       <c r="G20" s="11"/>
       <c r="H20" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I20" s="11"/>
       <c r="J20" s="12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="84">
       <c r="A21" s="13"/>
       <c r="B21" s="14"/>
       <c r="C21" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="E21" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="F21" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="G21" s="15" t="s">
         <v>112</v>
-      </c>
-      <c r="G21" s="15" t="s">
-        <v>113</v>
       </c>
       <c r="H21" s="11"/>
       <c r="I21" s="11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J21" s="11"/>
     </row>
@@ -1672,28 +1676,28 @@
         <v>10</v>
       </c>
       <c r="B22" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="D22" s="11" t="s">
         <v>116</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>117</v>
       </c>
       <c r="E22" s="11" t="s">
         <v>44</v>
       </c>
       <c r="F22" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="G22" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="G22" s="15" t="s">
+      <c r="H22" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="H22" s="11" t="s">
+      <c r="I22" s="11" t="s">
         <v>120</v>
-      </c>
-      <c r="I22" s="11" t="s">
-        <v>121</v>
       </c>
       <c r="J22" s="11"/>
     </row>
@@ -1701,19 +1705,19 @@
       <c r="A23" s="13"/>
       <c r="B23" s="14"/>
       <c r="C23" s="10" t="s">
+        <v>121</v>
+      </c>
+      <c r="D23" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="D23" s="11" t="s">
-        <v>123</v>
-      </c>
       <c r="E23" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F23" s="11"/>
       <c r="G23" s="11"/>
       <c r="H23" s="11"/>
       <c r="I23" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J23" s="11"/>
     </row>
@@ -1722,16 +1726,16 @@
         <v>11</v>
       </c>
       <c r="B24" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="C24" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="D24" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="E24" s="11" t="s">
         <v>127</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>87</v>
       </c>
       <c r="F24" s="11" t="s">
         <v>128</v>
@@ -1957,7 +1961,7 @@
         <v>176</v>
       </c>
       <c r="E33" s="11" t="s">
-        <v>87</v>
+        <v>127</v>
       </c>
       <c r="F33" s="11" t="s">
         <v>177</v>

</xml_diff>

<commit_message>
Publish course materials (be2b27ac)
Generated by scripts/publish_student.py from the source repository at be2b27ac: "Merge calendar-realign: weeks follow the calendar, Week 4 splits, HW6 gets real dates"
</commit_message>
<xml_diff>
--- a/schedule/CSCI3495_schedule_fall2026.xlsx
+++ b/schedule/CSCI3495_schedule_fall2026.xlsx
@@ -73,12 +73,12 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="007A7A7A"/>
-      <sz val="12"/>
+      <color rgb="007B341E"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="007B341E"/>
+      <color rgb="007A7A7A"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="7">
@@ -200,9 +200,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -212,11 +209,14 @@
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -822,38 +822,34 @@
       <c r="J6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Labor Day</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="A7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Python &amp; Data Science Foundations</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Mon Sep 7</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>No class</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr"/>
-      <c r="F7" s="13" t="inlineStr"/>
-      <c r="G7" s="13" t="inlineStr"/>
-      <c r="H7" s="13" t="inlineStr"/>
-      <c r="I7" s="13" t="inlineStr"/>
-      <c r="J7" s="13" t="inlineStr"/>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>No class, Labor Day</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr"/>
+      <c r="F7" s="12" t="inlineStr"/>
+      <c r="G7" s="12" t="inlineStr"/>
+      <c r="H7" s="12" t="inlineStr"/>
+      <c r="I7" s="12" t="inlineStr"/>
+      <c r="J7" s="12" t="inlineStr"/>
     </row>
     <row r="8" ht="84" customHeight="1">
-      <c r="A8" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Python &amp; Data Science Foundations</t>
-        </is>
-      </c>
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="8" t="n"/>
       <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Wed Sep 9</t>
@@ -861,12 +857,12 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Python for NLP: comprehensions and Counter; NumPy shape, dtype, broadcasting</t>
+          <t>Python, NumPy, pandas, seaborn, scikit-learn</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Lecture, Coding</t>
+          <t>Lecture</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -884,7 +880,11 @@
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr"/>
-      <c r="I8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>No class Mon Sep 7 (Labor Day), so this week meets once</t>
+        </is>
+      </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>Last day to opt Pass/Fail/Audit (Sep 11)</t>
@@ -892,8 +892,14 @@
       </c>
     </row>
     <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
+      <c r="A9" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Probability &amp; PyTorch</t>
+        </is>
+      </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Mon Sep 14</t>
@@ -901,37 +907,23 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>pandas &amp; PyTorch tensors: DataFrames, groupby, plotting; tensor shapes and autograd</t>
+          <t>Probability for NLP: joint, union, conditional, independence, Bayes</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Lecture, Quiz, Coding</t>
+          <t>Lecture, Whiteboard</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr"/>
       <c r="G9" s="6" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>HW1 released</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>Quiz 3</t>
-        </is>
-      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Vector Semantics &amp; Embeddings</t>
-        </is>
-      </c>
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
       <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Wed Sep 16</t>
@@ -939,7 +931,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Vector semantics: TF-IDF, PPMI, cosine similarity</t>
+          <t>PyTorch: tensors, dtype and shape, autograd, and the training loop</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -949,13 +941,23 @@
       </c>
       <c r="F10" s="6" t="inlineStr"/>
       <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>HW1 released</t>
+        </is>
+      </c>
       <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="6" t="inlineStr"/>
     </row>
-    <row r="11" ht="84" customHeight="1">
-      <c r="A11" s="8" t="n"/>
-      <c r="B11" s="8" t="n"/>
+    <row r="11" ht="58" customHeight="1">
+      <c r="A11" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Vector Semantics &amp; Embeddings</t>
+        </is>
+      </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Mon Sep 21</t>
@@ -963,689 +965,670 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
+          <t>Vector semantics: TF-IDF, PPMI, cosine similarity</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12" ht="84" customHeight="1">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Wed Sep 23</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
           <t>Word embeddings: word2vec, GloVe, analogies, embedding bias</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Lecture, Quiz, Whiteboard, Discussion</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Read word2vec (Mikolov 2013)</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=viZrOnJclY0
 https://www.youtube.com/watch?v=kEMJRjEdNzM</t>
         </is>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>HW1 due</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>Quiz 4</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>Early Alert grades due (Sep 23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="58" customHeight="1">
+      <c r="A13" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Neural Networks &amp; Sequence Models</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Wed Sep 23</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Mon Sep 28</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Neural networks for NLP: feedforward nets, training, backprop intuition</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Lecture, Coding, Whiteboard</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>HW2 released</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>Early Alert grades due (Sep 23)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="84" customHeight="1">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Mon Sep 28</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14" ht="84" customHeight="1">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Wed Sep 30</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>RNNs, LSTMs, vanishing gradients, language modeling</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>Lecture, Quiz, Coding</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Read seq2seq (Sutskever 2014)</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=YCzL96nL7j0
 https://www.youtube.com/watch?v=L8HKweZIOmg</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr"/>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Quiz 5</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15" ht="58" customHeight="1">
+      <c r="A15" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Attention &amp; the Transformer</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Wed Sep 30</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Mon Oct 5</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Seq2seq &amp; attention: encoder-decoder and the attention mechanism</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Lecture, Coding, Whiteboard</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr"/>
-      <c r="G14" s="6" t="inlineStr"/>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>HW2 due</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr"/>
-      <c r="J14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15" ht="70" customHeight="1">
-      <c r="A15" s="8" t="n"/>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Mon Oct 5</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16" ht="70" customHeight="1">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Wed Oct 7</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>The Transformer: self-attention, multi-head, positional encoding</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Lecture, Quiz, Coding</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Read 'Attention Is All You Need' (Vaswani 2017)</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=iDulhoQ2pro</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Project proposal due (submission only)</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Quiz 6</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16" ht="58" customHeight="1">
-      <c r="A16" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Pretraining &amp; BERT</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Wed Oct 7</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Mon Oct 12</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Contextual representations &amp; transfer learning: ELMo; pretrain→finetune</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Lecture, Discussion</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr"/>
-      <c r="G16" s="6" t="inlineStr"/>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr"/>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>HW3 released</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr"/>
-      <c r="J16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17" ht="70" customHeight="1">
-      <c r="A17" s="8" t="n"/>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Mon Oct 12</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Wed Oct 14</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>BERT &amp; masked language modeling: bidirectional pretraining, fine-tuning</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Lecture, Quiz, Coding</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Read BERT (Devlin 2019)</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=-9evrZnBorM</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr"/>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>Quiz 7</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr"/>
-    </row>
-    <row r="18" ht="70" customHeight="1">
-      <c r="A18" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>Class Recess, no university classes (Oct 16)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>LLMs: Generation &amp; Scaling</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Wed Oct 14</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Mon Oct 19</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>The GPT family &amp; autoregressive generation; decoding strategies</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Lecture, Coding, Discussion</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>Read GPT-3 (Brown 2020)</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>HW3 due</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20" ht="70" customHeight="1">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Wed Oct 21</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Scaling laws &amp; emergent abilities (Kaplan, Chinchilla)</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Lecture, Quiz, Whiteboard, Discussion</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr"/>
+      <c r="G20" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=_8yVOC4ciXc</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>HW3 due</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="inlineStr"/>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>Class Recess, no university classes (Oct 16)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Mon Oct 19</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Scaling laws &amp; emergent abilities (Kaplan, Chinchilla)</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Lecture, Quiz, Whiteboard, Discussion</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr"/>
-      <c r="G19" s="6" t="inlineStr"/>
-      <c r="H19" s="6" t="inlineStr"/>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Quiz 8</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="58" customHeight="1">
-      <c r="A20" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>Mid-term grades due (Oct 21)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Training &amp; Aligning LLMs</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Wed Oct 21</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Mon Oct 26</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Tokenization at scale (BPE); pretraining data &amp; compute; instruction tuning</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Lecture, Coding, Whiteboard</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr"/>
-      <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>HW4 released</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>Mid-term grades due (Oct 21)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="84" customHeight="1">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Mon Oct 26</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22" ht="84" customHeight="1">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Wed Oct 28</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
         <is>
           <t>Alignment: RLHF, InstructGPT, DPO; helpfulness vs. harmlessness</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>Lecture, Quiz, Discussion</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Read InstructGPT (Ouyang 2022)</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=iUZR0maBkOU
 https://www.youtube.com/watch?v=hvGa5Mba4c8</t>
         </is>
       </c>
-      <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr"/>
+      <c r="I22" s="6" t="inlineStr">
         <is>
           <t>Quiz 9</t>
         </is>
       </c>
-      <c r="J21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22" ht="70" customHeight="1">
-      <c r="A22" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="J22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="70" customHeight="1">
+      <c r="A23" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Efficiency &amp; Evaluation</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Wed Oct 28</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Mon Nov 2</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Efficient LLMs: LoRA/PEFT, quantization, running models locally</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>Lecture, Coding</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>Read LoRA (Hu 2021)</t>
         </is>
       </c>
-      <c r="G22" s="9" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=PXWYUTMt-AU</t>
         </is>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>HW4 due</t>
         </is>
       </c>
-      <c r="I22" s="6" t="inlineStr">
+      <c r="I23" s="6" t="inlineStr">
         <is>
           <t>Project work/feedback session (in-class)</t>
         </is>
       </c>
-      <c r="J22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="8" t="n"/>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Mon Nov 2</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="J23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Wed Nov 4</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Evaluation &amp; benchmarks: GLUE, MMLU, HELM, hallucination, contamination</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>Lecture, Quiz, Discussion</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr"/>
-      <c r="G23" s="6" t="inlineStr"/>
-      <c r="H23" s="6" t="inlineStr"/>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr">
         <is>
           <t>Quiz 10</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr"/>
-    </row>
-    <row r="24" ht="58" customHeight="1">
-      <c r="A24" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>Last day to withdraw from an undergraduate course (Nov 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Prompt Engineering</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Wed Nov 4</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Mon Nov 9</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>In-context learning &amp; prompt-engineering foundations: zero/few-shot</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>Lecture, Discussion</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Prepare the checkpoint talk</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr"/>
-      <c r="H24" s="6" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>HW5 released; Checkpoint due (10%)</t>
         </is>
       </c>
-      <c r="I24" s="6" t="inlineStr">
+      <c r="I25" s="6" t="inlineStr">
         <is>
           <t>Mid-semester checkpoint presentations</t>
         </is>
       </c>
-      <c r="J24" s="7" t="inlineStr">
-        <is>
-          <t>Last day to withdraw from an undergraduate course (Nov 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="84" customHeight="1">
-      <c r="A25" s="8" t="n"/>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Mon Nov 9</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>Pre-registration opens (Nov 9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="84" customHeight="1">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Wed Nov 11</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Advanced prompting: chain-of-thought, self-consistency, decomposition</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>Lecture, Quiz, Whiteboard, Discussion</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Read Chain-of-Thought (Wei 2022)</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=AFE6x81AP4k
 https://www.youtube.com/watch?v=DCqqCLlsIBU</t>
         </is>
       </c>
-      <c r="H25" s="6" t="inlineStr"/>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>Quiz 11</t>
         </is>
       </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>Pre-registration opens (Nov 9)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="58" customHeight="1">
-      <c r="A26" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="J26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27" ht="58" customHeight="1">
+      <c r="A27" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Structured Output &amp; RAG</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Wed Nov 11</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>MIDTERM EXAM (covers Weeks 1-11)</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Mon Nov 16</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>MIDTERM EXAM (covers Weeks 1-12)</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>Exam</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>Study for the midterm (study guide provided)</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr"/>
-      <c r="H26" s="6" t="inlineStr">
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>HW5 due</t>
         </is>
       </c>
-      <c r="I26" s="14" t="inlineStr">
+      <c r="I27" s="13" t="inlineStr">
         <is>
           <t>Midterm exam</t>
         </is>
       </c>
-      <c r="J26" s="6" t="inlineStr"/>
-    </row>
-    <row r="27" ht="70" customHeight="1">
-      <c r="A27" s="8" t="n"/>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Mon Nov 16</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="J27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28" ht="70" customHeight="1">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Wed Nov 18</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Retrieval-Augmented Generation (RAG): embeddings, vector search, grounding</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>Lecture, Quiz, Coding, Whiteboard</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>Read RAG (Lewis 2020)</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=JGpmQvlYRdU</t>
         </is>
       </c>
-      <c r="H27" s="6" t="inlineStr"/>
-      <c r="I27" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>HW6 released</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
         <is>
           <t>Quiz 12</t>
         </is>
       </c>
-      <c r="J27" s="6" t="inlineStr"/>
-    </row>
-    <row r="28" ht="84" customHeight="1">
-      <c r="A28" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Creating Agents</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Wed Nov 18</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>COMBINED SESSION: What is an LLM agent? ReAct, tool use, structured outputs, injection defense · The agent loop, memory and reflection; agent evaluation and failure modes, at surface level</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Lecture, Quiz, Coding, Discussion</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>Read ReAct (Yao 2022)</t>
-        </is>
-      </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Eug2clsLtFs
-https://www.youtube.com/watch?v=UID_oXuN-0Y</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>HW6 released · HW6 due</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>Quiz 13</t>
-        </is>
-      </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
           <t>Pre-registration closes (Nov 24)</t>
@@ -1653,56 +1636,56 @@
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="10" t="inlineStr"/>
-      <c r="B29" s="11" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr"/>
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>Thanksgiving Break</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>Mon Nov 23</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D29" s="11" t="inlineStr">
         <is>
           <t>No class</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr"/>
-      <c r="F29" s="13" t="inlineStr"/>
-      <c r="G29" s="13" t="inlineStr"/>
-      <c r="H29" s="13" t="inlineStr"/>
-      <c r="I29" s="13" t="inlineStr"/>
-      <c r="J29" s="13" t="inlineStr"/>
+      <c r="E29" s="12" t="inlineStr"/>
+      <c r="F29" s="12" t="inlineStr"/>
+      <c r="G29" s="12" t="inlineStr"/>
+      <c r="H29" s="12" t="inlineStr"/>
+      <c r="I29" s="12" t="inlineStr"/>
+      <c r="J29" s="12" t="inlineStr"/>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="15" t="n"/>
       <c r="B30" s="15" t="n"/>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C30" s="10" t="inlineStr">
         <is>
           <t>Wed Nov 25</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D30" s="11" t="inlineStr">
         <is>
           <t>No class</t>
         </is>
       </c>
-      <c r="E30" s="13" t="inlineStr"/>
-      <c r="F30" s="13" t="inlineStr"/>
-      <c r="G30" s="13" t="inlineStr"/>
-      <c r="H30" s="13" t="inlineStr"/>
-      <c r="I30" s="13" t="inlineStr"/>
-      <c r="J30" s="13" t="inlineStr"/>
-    </row>
-    <row r="31" ht="70" customHeight="1">
+      <c r="E30" s="12" t="inlineStr"/>
+      <c r="F30" s="12" t="inlineStr"/>
+      <c r="G30" s="12" t="inlineStr"/>
+      <c r="H30" s="12" t="inlineStr"/>
+      <c r="I30" s="12" t="inlineStr"/>
+      <c r="J30" s="12" t="inlineStr"/>
+    </row>
+    <row r="31" ht="84" customHeight="1">
       <c r="A31" s="3" t="n">
         <v>14</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Agentic Workflows</t>
+          <t>Agents &amp; Agentic Workflows</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -1712,99 +1695,108 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>COMBINED SESSION: Agentic workflows &amp; orchestration: chaining, routing, parallelization, multi-agent · Workflow patterns: reflection, evaluator-optimizer; when NOT to use agents</t>
+          <t>LLM agents: ReAct, tool use, structured output, injection defense, memory, reflection and evaluation</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
+          <t>Lecture, Coding, Discussion</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Read ReAct (Yao 2022)</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Eug2clsLtFs
+https://www.youtube.com/watch?v=UID_oXuN-0Y</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr"/>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>Deadline to apply for Spring 2027 graduation (Dec 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="70" customHeight="1">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Wed Dec 2</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Agentic workflows: chaining, routing, parallelization, multi-agent, reflection and evaluator-optimizer, and when NOT to use an agent</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
           <t>Lecture, Quiz, Coding, Discussion</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>Read 'Building Effective Agents' (Anthropic 2024)</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G32" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=LP5OCa20Zpg</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr"/>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="H32" s="6" t="inlineStr"/>
+      <c r="I32" s="6" t="inlineStr">
         <is>
           <t>Quiz 14; Project work/feedback (in-class)</t>
         </is>
       </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>Deadline to apply for Spring 2027 graduation (Dec 1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="70" customHeight="1">
-      <c r="A32" s="3" t="n">
+      <c r="J32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33" ht="70" customHeight="1">
+      <c r="A33" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Society, Ethics &amp; Wrap-up</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Wed Dec 2</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Ethics &amp; society: bias, fairness, 'Stochastic Parrots', misinformation, environment, copyright, safety</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Mon Dec 7</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>COMBINED SESSION: Ethics &amp; society: bias, fairness, 'Stochastic Parrots', misinformation, environment, copyright, safety · The future of NLP &amp; LLMs; course synthesis</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Lecture, Coding, Whiteboard, Discussion</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>Read Stochastic Parrots (Bender 2021)</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Read Stochastic Parrots (Bender 2021) · Prepare the final talk and report</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=WU4oou1GpCk</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr"/>
-      <c r="I32" s="6" t="inlineStr"/>
-      <c r="J32" s="6" t="inlineStr"/>
-    </row>
-    <row r="33" ht="58" customHeight="1">
-      <c r="A33" s="8" t="n"/>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Mon Dec 7</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>The future of NLP &amp; LLMs; course synthesis</t>
-        </is>
-      </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>Lecture, Discussion</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>Prepare the final talk and report</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr"/>
-      <c r="H33" s="6" t="inlineStr"/>
+      <c r="H33" s="6" t="inlineStr">
+        <is>
+          <t>HW6 due</t>
+        </is>
+      </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
           <t>Final presentations (Session 1)</t>
@@ -1865,60 +1857,58 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="B18:B19"/>
+  <mergeCells count="33">
+    <mergeCell ref="B27:B28"/>
     <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A28"/>
-    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="B33"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B11:B12"/>
     <mergeCell ref="B29:B30"/>
-    <mergeCell ref="A31"/>
-    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="A25:A26"/>
     <mergeCell ref="A3:A4"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B7"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B31"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="A21:A22"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="A7"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A13:A14"/>
     <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A19:A20"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="B28"/>
-    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="A33"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B31:B32"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Publish course materials (0a3c7b34)
Generated by scripts/publish_student.py from the source repository at 0a3c7b34: "Homeworks drive the schedule: real titles, and due dates that follow the lecture"
</commit_message>
<xml_diff>
--- a/schedule/CSCI3495_schedule_fall2026.xlsx
+++ b/schedule/CSCI3495_schedule_fall2026.xlsx
@@ -1422,11 +1422,7 @@
           <t>https://www.youtube.com/watch?v=PXWYUTMt-AU</t>
         </is>
       </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>HW4 due</t>
-        </is>
-      </c>
+      <c r="H23" s="6" t="inlineStr"/>
       <c r="I23" s="6" t="inlineStr">
         <is>
           <t>Project work/feedback session (in-class)</t>
@@ -1541,7 +1537,11 @@
 https://www.youtube.com/watch?v=DCqqCLlsIBU</t>
         </is>
       </c>
-      <c r="H26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>HW4 due</t>
+        </is>
+      </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
           <t>Quiz 11</t>
@@ -1579,11 +1579,7 @@
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr"/>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>HW5 due</t>
-        </is>
-      </c>
+      <c r="H27" s="6" t="inlineStr"/>
       <c r="I27" s="13" t="inlineStr">
         <is>
           <t>Midterm exam</t>
@@ -1714,7 +1710,11 @@
 https://www.youtube.com/watch?v=UID_oXuN-0Y</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr"/>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>HW5 due</t>
+        </is>
+      </c>
       <c r="I31" s="6" t="inlineStr"/>
       <c r="J31" s="7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Publish course materials (c06af686)
Generated by scripts/publish_student.py from the source repository at c06af686: "Drop the duplicate HW1 release from the PyTorch class"
</commit_message>
<xml_diff>
--- a/schedule/CSCI3495_schedule_fall2026.xlsx
+++ b/schedule/CSCI3495_schedule_fall2026.xlsx
@@ -941,11 +941,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr"/>
       <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>HW1 released</t>
-        </is>
-      </c>
+      <c r="H10" s="6" t="inlineStr"/>
       <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="6" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Publish course materials (27804a93)
Generated by scripts/publish_student.py from the source repository at 27804a93: "Readings: renumber for the two inserted weeks, and name the authority"
</commit_message>
<xml_diff>
--- a/schedule/CSCI3495_schedule_fall2026.xlsx
+++ b/schedule/CSCI3495_schedule_fall2026.xlsx
@@ -1011,7 +1011,7 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Quiz 4</t>
+          <t>Quiz 3</t>
         </is>
       </c>
       <c r="J12" s="7" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Lecture, Quiz, Coding</t>
+          <t>Lecture, Coding</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1084,11 +1084,7 @@
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr"/>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>Quiz 5</t>
-        </is>
-      </c>
+      <c r="I14" s="6" t="inlineStr"/>
       <c r="J14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="58" customHeight="1">
@@ -1160,7 +1156,7 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Quiz 6</t>
+          <t>Quiz 4</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr"/>
@@ -1214,7 +1210,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Lecture, Quiz, Coding</t>
+          <t>Lecture, Coding</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1228,11 +1224,7 @@
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr"/>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>Quiz 7</t>
-        </is>
-      </c>
+      <c r="I18" s="6" t="inlineStr"/>
       <c r="J18" s="7" t="inlineStr">
         <is>
           <t>Class Recess, no university classes (Oct 16)</t>
@@ -1304,7 +1296,7 @@
       <c r="H20" s="6" t="inlineStr"/>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Quiz 8</t>
+          <t>Quiz 5</t>
         </is>
       </c>
       <c r="J20" s="7" t="inlineStr">
@@ -1362,7 +1354,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Lecture, Quiz, Discussion</t>
+          <t>Lecture, Discussion</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1377,11 +1369,7 @@
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr"/>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>Quiz 9</t>
-        </is>
-      </c>
+      <c r="I22" s="6" t="inlineStr"/>
       <c r="J22" s="6" t="inlineStr"/>
     </row>
     <row r="23" ht="70" customHeight="1">
@@ -1449,7 +1437,7 @@
       <c r="H24" s="6" t="inlineStr"/>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>Quiz 10</t>
+          <t>Quiz 6</t>
         </is>
       </c>
       <c r="J24" s="7" t="inlineStr">
@@ -1519,7 +1507,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>Lecture, Quiz, Whiteboard, Discussion</t>
+          <t>Lecture, Whiteboard, Discussion</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -1538,11 +1526,7 @@
           <t>HW4 due</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>Quiz 11</t>
-        </is>
-      </c>
+      <c r="I26" s="6" t="inlineStr"/>
       <c r="J26" s="6" t="inlineStr"/>
     </row>
     <row r="27" ht="58" customHeight="1">
@@ -1618,7 +1602,7 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Quiz 12</t>
+          <t>Quiz 7</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
@@ -1733,7 +1717,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>Lecture, Quiz, Coding, Discussion</t>
+          <t>Lecture, Coding, Project Feedback</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -1749,7 +1733,7 @@
       <c r="H32" s="6" t="inlineStr"/>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>Quiz 14; Project work/feedback (in-class)</t>
+          <t>Project work/feedback (in-class)</t>
         </is>
       </c>
       <c r="J32" s="6" t="inlineStr"/>

</xml_diff>